<commit_message>
Add HMI WiFi setup flow
</commit_message>
<xml_diff>
--- a/Kaffeewaage.Logik.20250103.xlsx
+++ b/Kaffeewaage.Logik.20250103.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bernh\Documents\PlatformIO\Projects\KaffeewaageESP_SingleDose\KaffeewaageLilygoT-DisplayS3_20240212\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A2284C-B438-4A67-822F-834930045E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F11B8A-4F31-4EA4-A33E-9741DCDB480A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{6093FCE1-E198-4E7B-9A9F-5F65F14DDFBD}"/>
   </bookViews>
@@ -800,22 +800,6 @@
 pageID=8</t>
   </si>
   <si>
-    <r>
-      <t>Gefaess messen tara
-PageID</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>=9</t>
-    </r>
-  </si>
-  <si>
     <t>Reinigung Mühle
 pageID=11</t>
   </si>
@@ -830,10 +814,6 @@
   <si>
     <t>Daten 
 pageID=14</t>
-  </si>
-  <si>
-    <t>Gefaess messen Gefaess auflegen
-PageID=15</t>
   </si>
   <si>
     <r>
@@ -861,10 +841,6 @@
 pageID=18</t>
   </si>
   <si>
-    <t>Gefaess messen Gefaess gemessen
-pageID=23</t>
-  </si>
-  <si>
     <t>Pflege/Daten
 menuItemID=7</t>
   </si>
@@ -1163,6 +1139,30 @@
   </si>
   <si>
     <t>"Gefaess gemessen"</t>
+  </si>
+  <si>
+    <r>
+      <t>Gefaess messen, tara
+PageID</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>=9</t>
+    </r>
+  </si>
+  <si>
+    <t>Gefaess messen, Gefaess auflegen
+PageID=15</t>
+  </si>
+  <si>
+    <t>Gefaess messen, Gefaess gemessen
+pageID=23</t>
   </si>
 </sst>
 </file>
@@ -1577,7 +1577,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1712,12 +1712,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2752,8 +2746,8 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+    <row r="5" spans="1:7" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="49" t="s">
         <v>105</v>
       </c>
       <c r="B5" s="26" t="s">
@@ -2766,13 +2760,13 @@
         <v>228</v>
       </c>
       <c r="E5" s="48" t="s">
-        <v>231</v>
-      </c>
-      <c r="F5" s="49" t="s">
-        <v>236</v>
-      </c>
-      <c r="G5" s="50" t="s">
-        <v>240</v>
+        <v>307</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>308</v>
+      </c>
+      <c r="G5" s="48" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -2784,20 +2778,20 @@
         <v>219</v>
       </c>
       <c r="E6" s="45" t="s">
+        <v>254</v>
+      </c>
+      <c r="F6" s="46" t="s">
+        <v>256</v>
+      </c>
+      <c r="G6" s="31" t="s">
         <v>257</v>
-      </c>
-      <c r="F6" s="46" t="s">
-        <v>259</v>
-      </c>
-      <c r="G6" s="31" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="5"/>
       <c r="C7" s="10"/>
       <c r="D7" s="35" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E7" s="32" t="s">
         <v>209</v>
@@ -2813,7 +2807,7 @@
       <c r="B8" s="5"/>
       <c r="C8" s="10"/>
       <c r="D8" s="35" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E8" s="32" t="s">
         <v>212</v>
@@ -2829,7 +2823,7 @@
       <c r="B9" s="5"/>
       <c r="C9" s="10"/>
       <c r="D9" s="35" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E9" s="32" t="s">
         <v>215</v>
@@ -2844,14 +2838,14 @@
     <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="5"/>
       <c r="C10" s="10"/>
-      <c r="D10" s="52" t="s">
+      <c r="D10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="E10" s="52" t="s">
+      <c r="E10" s="50" t="s">
         <v>221</v>
       </c>
-      <c r="F10" s="52" t="s">
-        <v>237</v>
+      <c r="F10" s="50" t="s">
+        <v>235</v>
       </c>
       <c r="G10" s="25"/>
     </row>
@@ -2861,10 +2855,10 @@
         <v>135</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F11" s="30" t="s">
         <v>188</v>
@@ -2874,8 +2868,8 @@
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B12" s="36"/>
       <c r="C12" s="39"/>
-      <c r="D12" s="53" t="s">
-        <v>278</v>
+      <c r="D12" s="51" t="s">
+        <v>275</v>
       </c>
       <c r="E12" s="40"/>
       <c r="F12" s="37"/>
@@ -2887,7 +2881,7 @@
         <v>218</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E13" s="39"/>
       <c r="G13" s="34"/>
@@ -2896,7 +2890,7 @@
       <c r="B14" s="36"/>
       <c r="C14" s="41"/>
       <c r="D14" s="35" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E14" s="39"/>
       <c r="G14" s="34"/>
@@ -2904,16 +2898,16 @@
     <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B15" s="36"/>
       <c r="C15" s="35" t="s">
-        <v>241</v>
-      </c>
-      <c r="D15" s="53" t="s">
+        <v>238</v>
+      </c>
+      <c r="D15" s="51" t="s">
         <v>230</v>
       </c>
-      <c r="E15" s="53" t="s">
-        <v>232</v>
-      </c>
-      <c r="F15" s="53" t="s">
-        <v>238</v>
+      <c r="E15" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>236</v>
       </c>
       <c r="G15" s="34"/>
     </row>
@@ -2921,7 +2915,7 @@
       <c r="B16" s="36"/>
       <c r="C16" s="39"/>
       <c r="D16" s="35" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E16" s="35" t="s">
         <v>194</v>
@@ -2935,11 +2929,11 @@
       <c r="B17" s="36"/>
       <c r="C17" s="41"/>
       <c r="D17" s="39"/>
-      <c r="E17" s="53" t="s">
-        <v>233</v>
-      </c>
-      <c r="F17" s="53" t="s">
-        <v>239</v>
+      <c r="E17" s="51" t="s">
+        <v>232</v>
+      </c>
+      <c r="F17" s="51" t="s">
+        <v>237</v>
       </c>
       <c r="G17" s="34"/>
     </row>
@@ -2947,7 +2941,7 @@
       <c r="B18" s="36"/>
       <c r="C18" s="41"/>
       <c r="D18" s="35" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E18" s="35" t="s">
         <v>194</v>
@@ -2961,10 +2955,10 @@
       <c r="B19" s="36"/>
       <c r="C19" s="41"/>
       <c r="D19" s="39"/>
-      <c r="E19" s="53" t="s">
-        <v>234</v>
-      </c>
-      <c r="F19" s="53" t="s">
+      <c r="E19" s="51" t="s">
+        <v>233</v>
+      </c>
+      <c r="F19" s="51" t="s">
         <v>200</v>
       </c>
       <c r="G19" s="34"/>
@@ -2973,7 +2967,7 @@
       <c r="B20" s="36"/>
       <c r="C20" s="41"/>
       <c r="D20" s="35" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E20" s="35" t="s">
         <v>194</v>
@@ -2987,10 +2981,10 @@
       <c r="B21" s="36"/>
       <c r="C21" s="41"/>
       <c r="D21" s="39"/>
-      <c r="E21" s="53" t="s">
-        <v>235</v>
-      </c>
-      <c r="F21" s="53" t="s">
+      <c r="E21" s="51" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="51" t="s">
         <v>222</v>
       </c>
       <c r="G21" s="34"/>
@@ -2999,7 +2993,7 @@
       <c r="B22" s="36"/>
       <c r="C22" s="42"/>
       <c r="D22" s="35" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E22" s="35" t="s">
         <v>204</v>
@@ -3011,40 +3005,40 @@
     </row>
     <row r="23" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B23" s="36"/>
-      <c r="C23" s="58"/>
+      <c r="C23" s="56"/>
       <c r="D23" s="41"/>
       <c r="E23" s="41"/>
-      <c r="F23" s="53" t="s">
+      <c r="F23" s="51" t="s">
         <v>223</v>
       </c>
       <c r="G23" s="34"/>
     </row>
     <row r="24" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B24" s="36"/>
-      <c r="C24" s="58"/>
+      <c r="C24" s="56"/>
       <c r="D24" s="41"/>
       <c r="E24" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="F24" s="59" t="s">
+      <c r="F24" s="57" t="s">
         <v>206</v>
       </c>
       <c r="G24" s="34"/>
     </row>
     <row r="25" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="58"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="56"/>
       <c r="E25" s="41"/>
-      <c r="F25" s="53" t="s">
+      <c r="F25" s="51" t="s">
         <v>224</v>
       </c>
       <c r="G25" s="34"/>
     </row>
     <row r="26" spans="2:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="36"/>
-      <c r="C26" s="58"/>
-      <c r="D26" s="58"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
       <c r="E26" s="35" t="s">
         <v>207</v>
       </c>
@@ -3057,7 +3051,7 @@
       <c r="B27" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="C27" s="53" t="s">
+      <c r="C27" s="51" t="s">
         <v>111</v>
       </c>
       <c r="D27" s="4"/>
@@ -3068,7 +3062,7 @@
     <row r="28" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B28" s="6"/>
       <c r="C28" s="43" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="11"/>
@@ -3078,7 +3072,7 @@
     <row r="29" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B29" s="6"/>
       <c r="C29" s="43" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="11"/>
@@ -3088,7 +3082,7 @@
     <row r="30" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B30" s="6"/>
       <c r="C30" s="43" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="11"/>
@@ -3098,7 +3092,7 @@
     <row r="31" spans="2:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6"/>
       <c r="C31" s="29" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="14"/>
@@ -3109,7 +3103,7 @@
       <c r="B32" s="27" t="s">
         <v>225</v>
       </c>
-      <c r="C32" s="53" t="s">
+      <c r="C32" s="51" t="s">
         <v>226</v>
       </c>
       <c r="D32" s="9"/>
@@ -3121,7 +3115,7 @@
       <c r="B33" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="C33" s="53" t="s">
+      <c r="C33" s="51" t="s">
         <v>227</v>
       </c>
       <c r="D33" s="9"/>
@@ -3132,7 +3126,7 @@
     <row r="34" spans="2:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="7"/>
       <c r="C34" s="29" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
@@ -3236,13 +3230,13 @@
         <v>80</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>81</v>
@@ -3274,7 +3268,7 @@
         <v>83</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H7" s="18"/>
     </row>
@@ -3304,13 +3298,13 @@
         <v>80</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>85</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H9" s="18"/>
     </row>
@@ -3336,7 +3330,7 @@
         <v>87</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="H11" s="18"/>
     </row>
@@ -3349,7 +3343,7 @@
         <v>88</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="H12" s="18"/>
     </row>
@@ -3364,13 +3358,13 @@
         <v>80</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H13" s="18"/>
     </row>
@@ -3379,19 +3373,19 @@
         <v>83</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H14" s="18"/>
     </row>
@@ -3400,19 +3394,19 @@
         <v>84</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D15" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H15" s="18"/>
     </row>
@@ -3421,7 +3415,7 @@
         <v>85</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>81</v>
@@ -3433,7 +3427,7 @@
         <v>89</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="H16" s="18"/>
     </row>
@@ -3454,7 +3448,7 @@
         <v>90</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="H17" s="18"/>
     </row>
@@ -3463,7 +3457,7 @@
         <v>87</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D18" s="19" t="s">
         <v>81</v>
@@ -3475,7 +3469,7 @@
         <v>80</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H18" s="18"/>
     </row>
@@ -3484,7 +3478,7 @@
         <v>88</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>81</v>
@@ -3496,7 +3490,7 @@
         <v>91</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H19" s="18"/>
     </row>
@@ -3544,19 +3538,19 @@
         <v>89</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D23" s="19" t="s">
         <v>85</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>191</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H23" s="18"/>
     </row>
@@ -3565,7 +3559,7 @@
         <v>90</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>86</v>
@@ -3586,19 +3580,19 @@
         <v>91</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>88</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>193</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H25" s="18"/>
     </row>
@@ -3613,10 +3607,10 @@
         <v>88</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>187</v>
@@ -3634,10 +3628,10 @@
         <v>88</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>186</v>
@@ -3655,10 +3649,10 @@
         <v>88</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>204</v>
@@ -3671,7 +3665,7 @@
       <c r="D29" s="19"/>
       <c r="E29" s="20"/>
       <c r="F29" s="4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="G29" s="4" t="s">
         <v>205</v>
@@ -3684,7 +3678,7 @@
       <c r="D30" s="19"/>
       <c r="E30" s="20"/>
       <c r="F30" s="19" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>207</v>
@@ -3696,19 +3690,19 @@
         <v>191</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D31" s="19" t="s">
         <v>89</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="H31" s="18"/>
     </row>
@@ -3723,13 +3717,13 @@
         <v>90</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F32" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H32" s="4"/>
     </row>
@@ -3738,25 +3732,25 @@
         <v>193</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>91</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="F33" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B34" s="19" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>187</v>
@@ -3771,13 +3765,13 @@
         <v>80</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H34" s="4"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B35" s="19" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>186</v>
@@ -3792,13 +3786,13 @@
         <v>80</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B36" s="4" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>204</v>
@@ -3813,13 +3807,13 @@
         <v>80</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H36" s="4"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B37" s="4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>205</v>
@@ -3834,13 +3828,13 @@
         <v>80</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B38" s="19" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>207</v>
@@ -3855,28 +3849,28 @@
         <v>80</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H38" s="4"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B39" s="4" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D39" s="19" t="s">
         <v>191</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F39" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G39" s="20" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H39" s="4"/>
     </row>
@@ -4011,7 +4005,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="24" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C51" s="24"/>
       <c r="G51" s="24"/>
@@ -4044,7 +4038,7 @@
         <v>3</v>
       </c>
       <c r="B54" s="24" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C54" s="24"/>
       <c r="G54" s="24"/>
@@ -4054,7 +4048,7 @@
         <v>4</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C55" s="24"/>
       <c r="G55" s="24"/>
@@ -4064,7 +4058,7 @@
         <v>5</v>
       </c>
       <c r="B56" s="24" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C56" s="24"/>
       <c r="G56" s="24"/>
@@ -4084,7 +4078,7 @@
         <v>7</v>
       </c>
       <c r="B58" s="24" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C58" s="24"/>
       <c r="G58" s="24"/>
@@ -4094,7 +4088,7 @@
         <v>8</v>
       </c>
       <c r="B59" s="24" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C59" s="24"/>
       <c r="G59" s="24"/>
@@ -4104,7 +4098,7 @@
         <v>9</v>
       </c>
       <c r="B60" s="24" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C60" s="24"/>
       <c r="G60" s="24"/>
@@ -4163,7 +4157,7 @@
         <v>15</v>
       </c>
       <c r="B66" s="24" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C66" s="24"/>
       <c r="G66" s="24"/>
@@ -4243,26 +4237,26 @@
         <v>23</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C74" s="24"/>
       <c r="G74" s="24"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="24"/>
-      <c r="B75" s="55"/>
+      <c r="B75" s="53"/>
       <c r="C75" s="24"/>
       <c r="G75" s="24"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="24"/>
-      <c r="B76" s="55"/>
+      <c r="B76" s="53"/>
       <c r="C76" s="24"/>
       <c r="G76" s="24"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="24"/>
-      <c r="B77" s="55"/>
+      <c r="B77" s="53"/>
       <c r="C77" s="24"/>
       <c r="G77" s="24"/>
     </row>
@@ -4294,7 +4288,7 @@
         <v>72</v>
       </c>
       <c r="D81" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E81" s="24" t="s">
         <v>126</v>
@@ -4305,17 +4299,17 @@
       <c r="A82" s="24">
         <v>1</v>
       </c>
-      <c r="B82" s="62" t="s">
-        <v>281</v>
-      </c>
-      <c r="C82" s="62" t="s">
+      <c r="B82" s="60" t="s">
+        <v>278</v>
+      </c>
+      <c r="C82" s="60" t="s">
         <v>127</v>
       </c>
-      <c r="D82" s="60" t="s">
-        <v>282</v>
-      </c>
-      <c r="E82" s="62" t="s">
-        <v>283</v>
+      <c r="D82" s="58" t="s">
+        <v>279</v>
+      </c>
+      <c r="E82" s="60" t="s">
+        <v>280</v>
       </c>
       <c r="G82" s="24"/>
     </row>
@@ -4323,17 +4317,17 @@
       <c r="A83" s="24">
         <v>2</v>
       </c>
-      <c r="B83" s="60" t="s">
+      <c r="B83" s="58" t="s">
         <v>129</v>
       </c>
-      <c r="C83" s="60" t="s">
-        <v>288</v>
-      </c>
-      <c r="D83" s="60" t="s">
-        <v>289</v>
-      </c>
-      <c r="E83" s="60" t="s">
-        <v>290</v>
+      <c r="C83" s="58" t="s">
+        <v>285</v>
+      </c>
+      <c r="D83" s="58" t="s">
+        <v>286</v>
+      </c>
+      <c r="E83" s="58" t="s">
+        <v>287</v>
       </c>
       <c r="G83" s="24"/>
     </row>
@@ -4341,16 +4335,16 @@
       <c r="A84" s="24">
         <v>3</v>
       </c>
-      <c r="B84" s="62" t="s">
+      <c r="B84" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="C84" s="62" t="s">
+      <c r="C84" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="D84" s="60" t="s">
+      <c r="D84" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="E84" s="62" t="s">
+      <c r="E84" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G84" s="24"/>
@@ -4359,16 +4353,16 @@
       <c r="A85" s="24">
         <v>4</v>
       </c>
-      <c r="B85" s="62" t="s">
+      <c r="B85" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="C85" s="62" t="s">
+      <c r="C85" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="D85" s="60" t="s">
-        <v>262</v>
-      </c>
-      <c r="E85" s="62" t="s">
+      <c r="D85" s="58" t="s">
+        <v>259</v>
+      </c>
+      <c r="E85" s="60" t="s">
         <v>126</v>
       </c>
       <c r="G85" s="24"/>
@@ -4377,17 +4371,17 @@
       <c r="A86" s="24">
         <v>5</v>
       </c>
-      <c r="B86" s="62" t="s">
+      <c r="B86" s="60" t="s">
+        <v>281</v>
+      </c>
+      <c r="C86" s="60" t="s">
         <v>284</v>
       </c>
-      <c r="C86" s="62" t="s">
-        <v>287</v>
-      </c>
-      <c r="D86" s="60" t="s">
-        <v>285</v>
-      </c>
-      <c r="E86" s="62" t="s">
-        <v>286</v>
+      <c r="D86" s="58" t="s">
+        <v>282</v>
+      </c>
+      <c r="E86" s="60" t="s">
+        <v>283</v>
       </c>
       <c r="G86" s="24"/>
     </row>
@@ -4395,16 +4389,16 @@
       <c r="A87" s="24">
         <v>6</v>
       </c>
-      <c r="B87" s="62" t="s">
+      <c r="B87" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="C87" s="62" t="s">
+      <c r="C87" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="D87" s="62" t="s">
+      <c r="D87" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E87" s="60" t="s">
+      <c r="E87" s="58" t="s">
         <v>128</v>
       </c>
       <c r="G87" s="24"/>
@@ -4413,16 +4407,16 @@
       <c r="A88" s="24">
         <v>7</v>
       </c>
-      <c r="B88" s="62" t="s">
-        <v>292</v>
-      </c>
-      <c r="C88" s="62" t="s">
-        <v>293</v>
-      </c>
-      <c r="D88" s="62" t="s">
+      <c r="B88" s="60" t="s">
+        <v>289</v>
+      </c>
+      <c r="C88" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="D88" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E88" s="60" t="s">
+      <c r="E88" s="58" t="s">
         <v>128</v>
       </c>
       <c r="G88" s="24"/>
@@ -4431,16 +4425,16 @@
       <c r="A89" s="24">
         <v>8</v>
       </c>
-      <c r="B89" s="63" t="s">
+      <c r="B89" s="61" t="s">
         <v>197</v>
       </c>
-      <c r="C89" s="62" t="s">
+      <c r="C89" s="60" t="s">
         <v>198</v>
       </c>
-      <c r="D89" s="62" t="s">
+      <c r="D89" s="60" t="s">
         <v>199</v>
       </c>
-      <c r="E89" s="60" t="s">
+      <c r="E89" s="58" t="s">
         <v>195</v>
       </c>
       <c r="G89" s="24"/>
@@ -4449,16 +4443,16 @@
       <c r="A90" s="24">
         <v>9</v>
       </c>
-      <c r="B90" s="62" t="s">
-        <v>294</v>
-      </c>
-      <c r="C90" s="62" t="s">
+      <c r="B90" s="60" t="s">
+        <v>291</v>
+      </c>
+      <c r="C90" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="D90" s="62" t="s">
+      <c r="D90" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E90" s="60" t="s">
+      <c r="E90" s="58" t="s">
         <v>128</v>
       </c>
       <c r="G90" s="24"/>
@@ -4467,16 +4461,16 @@
       <c r="A91" s="24">
         <v>10</v>
       </c>
-      <c r="B91" s="62" t="s">
-        <v>301</v>
-      </c>
-      <c r="C91" s="62" t="s">
-        <v>302</v>
-      </c>
-      <c r="D91" s="62" t="s">
+      <c r="B91" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="C91" s="60" t="s">
+        <v>299</v>
+      </c>
+      <c r="D91" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E91" s="60" t="s">
+      <c r="E91" s="58" t="s">
         <v>128</v>
       </c>
       <c r="G91" s="24"/>
@@ -4485,16 +4479,16 @@
       <c r="A92" s="24">
         <v>11</v>
       </c>
-      <c r="B92" s="62" t="s">
-        <v>295</v>
-      </c>
-      <c r="C92" s="62" t="s">
+      <c r="B92" s="60" t="s">
+        <v>292</v>
+      </c>
+      <c r="C92" s="60" t="s">
         <v>196</v>
       </c>
-      <c r="D92" s="62" t="s">
+      <c r="D92" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E92" s="62" t="s">
+      <c r="E92" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G92" s="24"/>
@@ -4503,16 +4497,16 @@
       <c r="A93" s="24">
         <v>12</v>
       </c>
-      <c r="B93" s="62" t="s">
-        <v>295</v>
-      </c>
-      <c r="C93" s="62" t="s">
+      <c r="B93" s="60" t="s">
+        <v>292</v>
+      </c>
+      <c r="C93" s="60" t="s">
         <v>196</v>
       </c>
-      <c r="D93" s="62" t="s">
+      <c r="D93" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E93" s="62" t="s">
+      <c r="E93" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G93" s="24"/>
@@ -4521,30 +4515,30 @@
       <c r="A94" s="24">
         <v>13</v>
       </c>
-      <c r="B94" s="62" t="s">
-        <v>296</v>
-      </c>
-      <c r="C94" s="62" t="s">
+      <c r="B94" s="60" t="s">
+        <v>293</v>
+      </c>
+      <c r="C94" s="60" t="s">
         <v>196</v>
       </c>
-      <c r="D94" s="60"/>
-      <c r="E94" s="60"/>
+      <c r="D94" s="58"/>
+      <c r="E94" s="58"/>
       <c r="G94" s="24"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="24">
         <v>14</v>
       </c>
-      <c r="B95" s="62" t="s">
-        <v>297</v>
-      </c>
-      <c r="C95" s="62" t="s">
-        <v>298</v>
-      </c>
-      <c r="D95" s="62" t="s">
-        <v>299</v>
-      </c>
-      <c r="E95" s="62" t="s">
+      <c r="B95" s="60" t="s">
+        <v>294</v>
+      </c>
+      <c r="C95" s="60" t="s">
+        <v>295</v>
+      </c>
+      <c r="D95" s="60" t="s">
+        <v>296</v>
+      </c>
+      <c r="E95" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G95" s="24"/>
@@ -4553,16 +4547,16 @@
       <c r="A96" s="24">
         <v>15</v>
       </c>
-      <c r="B96" s="62" t="s">
-        <v>294</v>
-      </c>
-      <c r="C96" s="62" t="s">
-        <v>300</v>
-      </c>
-      <c r="D96" s="62" t="s">
+      <c r="B96" s="60" t="s">
+        <v>291</v>
+      </c>
+      <c r="C96" s="60" t="s">
+        <v>297</v>
+      </c>
+      <c r="D96" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E96" s="62" t="s">
+      <c r="E96" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G96" s="24"/>
@@ -4571,16 +4565,16 @@
       <c r="A97" s="24">
         <v>16</v>
       </c>
-      <c r="B97" s="62" t="s">
-        <v>305</v>
-      </c>
-      <c r="C97" s="62" t="s">
+      <c r="B97" s="60" t="s">
+        <v>302</v>
+      </c>
+      <c r="C97" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="D97" s="60" t="s">
+      <c r="D97" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="E97" s="62" t="s">
+      <c r="E97" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G97" s="24"/>
@@ -4589,16 +4583,16 @@
       <c r="A98" s="24">
         <v>17</v>
       </c>
-      <c r="B98" s="64" t="s">
-        <v>303</v>
-      </c>
-      <c r="C98" s="62" t="s">
+      <c r="B98" s="62" t="s">
+        <v>300</v>
+      </c>
+      <c r="C98" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="D98" s="62" t="s">
+      <c r="D98" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E98" s="62" t="s">
+      <c r="E98" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G98" s="24"/>
@@ -4607,16 +4601,16 @@
       <c r="A99" s="24">
         <v>18</v>
       </c>
-      <c r="B99" s="64" t="s">
-        <v>304</v>
-      </c>
-      <c r="C99" s="62" t="s">
+      <c r="B99" s="62" t="s">
+        <v>301</v>
+      </c>
+      <c r="C99" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="D99" s="62" t="s">
+      <c r="D99" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E99" s="62" t="s">
+      <c r="E99" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G99" s="24"/>
@@ -4625,16 +4619,16 @@
       <c r="A100" s="24">
         <v>19</v>
       </c>
-      <c r="B100" s="64" t="s">
-        <v>306</v>
-      </c>
-      <c r="C100" s="62" t="s">
+      <c r="B100" s="62" t="s">
+        <v>303</v>
+      </c>
+      <c r="C100" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="D100" s="62" t="s">
+      <c r="D100" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E100" s="62" t="s">
+      <c r="E100" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G100" s="24"/>
@@ -4643,16 +4637,16 @@
       <c r="A101" s="24">
         <v>20</v>
       </c>
-      <c r="B101" s="64" t="s">
-        <v>307</v>
-      </c>
-      <c r="C101" s="62" t="s">
-        <v>308</v>
-      </c>
-      <c r="D101" s="62" t="s">
+      <c r="B101" s="62" t="s">
+        <v>304</v>
+      </c>
+      <c r="C101" s="60" t="s">
+        <v>305</v>
+      </c>
+      <c r="D101" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="E101" s="62" t="s">
+      <c r="E101" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G101" s="24"/>
@@ -4661,16 +4655,16 @@
       <c r="A102" s="24">
         <v>21</v>
       </c>
-      <c r="B102" s="64" t="s">
-        <v>307</v>
-      </c>
-      <c r="C102" s="62" t="s">
-        <v>308</v>
-      </c>
-      <c r="D102" s="62" t="s">
+      <c r="B102" s="62" t="s">
+        <v>304</v>
+      </c>
+      <c r="C102" s="60" t="s">
+        <v>305</v>
+      </c>
+      <c r="D102" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="E102" s="62" t="s">
+      <c r="E102" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G102" s="24"/>
@@ -4679,16 +4673,16 @@
       <c r="A103" s="24">
         <v>22</v>
       </c>
-      <c r="B103" s="64" t="s">
-        <v>299</v>
-      </c>
-      <c r="C103" s="62" t="s">
+      <c r="B103" s="62" t="s">
+        <v>296</v>
+      </c>
+      <c r="C103" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="D103" s="62" t="s">
+      <c r="D103" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="E103" s="62" t="s">
+      <c r="E103" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G103" s="24"/>
@@ -4697,25 +4691,25 @@
       <c r="A104" s="24">
         <v>23</v>
       </c>
-      <c r="B104" s="62" t="s">
-        <v>294</v>
-      </c>
-      <c r="C104" s="62" t="s">
-        <v>309</v>
-      </c>
-      <c r="D104" s="62" t="s">
+      <c r="B104" s="60" t="s">
+        <v>291</v>
+      </c>
+      <c r="C104" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="D104" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="E104" s="62" t="s">
+      <c r="E104" s="60" t="s">
         <v>128</v>
       </c>
       <c r="G104" s="24"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B105" s="62"/>
-      <c r="C105" s="62"/>
-      <c r="D105" s="62"/>
-      <c r="E105" s="62"/>
+      <c r="B105" s="60"/>
+      <c r="C105" s="60"/>
+      <c r="D105" s="60"/>
+      <c r="E105" s="60"/>
       <c r="G105" s="24"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
@@ -4741,7 +4735,7 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="G108" s="24"/>
     </row>
@@ -4765,7 +4759,7 @@
         <v>1</v>
       </c>
       <c r="D110" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="G110" s="24"/>
     </row>
@@ -4865,7 +4859,7 @@
       <c r="A121" s="24">
         <v>13</v>
       </c>
-      <c r="B121" s="62">
+      <c r="B121" s="60">
         <v>1</v>
       </c>
       <c r="C121" s="24"/>
@@ -4875,7 +4869,7 @@
       <c r="A122" s="24">
         <v>14</v>
       </c>
-      <c r="B122" s="62">
+      <c r="B122" s="60">
         <v>1</v>
       </c>
       <c r="C122" s="24"/>
@@ -4885,7 +4879,7 @@
       <c r="A123" s="24">
         <v>15</v>
       </c>
-      <c r="B123" s="62">
+      <c r="B123" s="60">
         <v>1</v>
       </c>
       <c r="C123" s="24"/>
@@ -4895,7 +4889,7 @@
       <c r="A124" s="24">
         <v>16</v>
       </c>
-      <c r="B124" s="62">
+      <c r="B124" s="60">
         <v>1</v>
       </c>
       <c r="C124" s="24"/>
@@ -4905,7 +4899,7 @@
       <c r="A125" s="24">
         <v>17</v>
       </c>
-      <c r="B125" s="62">
+      <c r="B125" s="60">
         <v>1</v>
       </c>
       <c r="C125" s="24"/>
@@ -4915,7 +4909,7 @@
       <c r="A126" s="24">
         <v>18</v>
       </c>
-      <c r="B126" s="62">
+      <c r="B126" s="60">
         <v>1</v>
       </c>
       <c r="C126" s="24"/>
@@ -4925,7 +4919,7 @@
       <c r="A127" s="24">
         <v>19</v>
       </c>
-      <c r="B127" s="62">
+      <c r="B127" s="60">
         <v>1</v>
       </c>
       <c r="C127" s="24"/>
@@ -4935,7 +4929,7 @@
       <c r="A128" s="24">
         <v>20</v>
       </c>
-      <c r="B128" s="62">
+      <c r="B128" s="60">
         <v>1</v>
       </c>
       <c r="C128" s="24"/>
@@ -4945,7 +4939,7 @@
       <c r="A129" s="24">
         <v>21</v>
       </c>
-      <c r="B129" s="62">
+      <c r="B129" s="60">
         <v>1</v>
       </c>
       <c r="C129" s="24"/>
@@ -4955,7 +4949,7 @@
       <c r="A130" s="24">
         <v>22</v>
       </c>
-      <c r="B130" s="62">
+      <c r="B130" s="60">
         <v>1</v>
       </c>
       <c r="C130" s="24"/>
@@ -4965,7 +4959,7 @@
       <c r="A131" s="24">
         <v>23</v>
       </c>
-      <c r="B131" s="62">
+      <c r="B131" s="60">
         <v>1</v>
       </c>
       <c r="C131" s="24"/>
@@ -4973,7 +4967,7 @@
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132" s="24"/>
-      <c r="B132" s="54"/>
+      <c r="B132" s="52"/>
       <c r="C132" s="24"/>
       <c r="G132" s="24"/>
     </row>
@@ -5125,7 +5119,7 @@
       <c r="A148" s="24">
         <v>13</v>
       </c>
-      <c r="B148" s="62">
+      <c r="B148" s="60">
         <v>0</v>
       </c>
       <c r="C148" s="24"/>
@@ -5135,7 +5129,7 @@
       <c r="A149" s="24">
         <v>14</v>
       </c>
-      <c r="B149" s="62">
+      <c r="B149" s="60">
         <v>0</v>
       </c>
       <c r="C149" s="24"/>
@@ -5145,7 +5139,7 @@
       <c r="A150" s="24">
         <v>15</v>
       </c>
-      <c r="B150" s="62">
+      <c r="B150" s="60">
         <v>1</v>
       </c>
       <c r="C150" s="24"/>
@@ -5155,7 +5149,7 @@
       <c r="A151" s="24">
         <v>16</v>
       </c>
-      <c r="B151" s="62">
+      <c r="B151" s="60">
         <v>1</v>
       </c>
       <c r="C151" s="24"/>
@@ -5165,7 +5159,7 @@
       <c r="A152" s="24">
         <v>17</v>
       </c>
-      <c r="B152" s="62">
+      <c r="B152" s="60">
         <v>0</v>
       </c>
       <c r="C152" s="24"/>
@@ -5175,7 +5169,7 @@
       <c r="A153" s="24">
         <v>18</v>
       </c>
-      <c r="B153" s="62">
+      <c r="B153" s="60">
         <v>0</v>
       </c>
       <c r="C153" s="24"/>
@@ -5185,7 +5179,7 @@
       <c r="A154" s="24">
         <v>19</v>
       </c>
-      <c r="B154" s="62">
+      <c r="B154" s="60">
         <v>0</v>
       </c>
       <c r="C154" s="24"/>
@@ -5195,7 +5189,7 @@
       <c r="A155" s="24">
         <v>20</v>
       </c>
-      <c r="B155" s="62">
+      <c r="B155" s="60">
         <v>0</v>
       </c>
       <c r="C155" s="24"/>
@@ -5205,7 +5199,7 @@
       <c r="A156" s="24">
         <v>21</v>
       </c>
-      <c r="B156" s="62">
+      <c r="B156" s="60">
         <v>0</v>
       </c>
       <c r="C156" s="24"/>
@@ -5215,7 +5209,7 @@
       <c r="A157" s="24">
         <v>22</v>
       </c>
-      <c r="B157" s="62">
+      <c r="B157" s="60">
         <v>0</v>
       </c>
       <c r="C157" s="24"/>
@@ -5225,7 +5219,7 @@
       <c r="A158" s="24">
         <v>23</v>
       </c>
-      <c r="B158" s="62">
+      <c r="B158" s="60">
         <v>1</v>
       </c>
       <c r="C158" s="24"/>
@@ -5395,7 +5389,7 @@
       <c r="A176" s="24">
         <v>13</v>
       </c>
-      <c r="B176" s="61">
+      <c r="B176" s="59">
         <v>8</v>
       </c>
       <c r="C176" s="24"/>
@@ -5405,7 +5399,7 @@
       <c r="A177" s="24">
         <v>14</v>
       </c>
-      <c r="B177" s="61">
+      <c r="B177" s="59">
         <v>8</v>
       </c>
       <c r="C177" s="24"/>
@@ -5415,7 +5409,7 @@
       <c r="A178" s="24">
         <v>15</v>
       </c>
-      <c r="B178" s="61">
+      <c r="B178" s="59">
         <v>9</v>
       </c>
       <c r="C178" s="24"/>
@@ -5425,7 +5419,7 @@
       <c r="A179" s="24">
         <v>16</v>
       </c>
-      <c r="B179" s="61">
+      <c r="B179" s="59">
         <v>10</v>
       </c>
       <c r="C179" s="24"/>
@@ -5435,7 +5429,7 @@
       <c r="A180" s="24">
         <v>17</v>
       </c>
-      <c r="B180" s="61">
+      <c r="B180" s="59">
         <v>11</v>
       </c>
       <c r="C180" s="24"/>
@@ -5445,7 +5439,7 @@
       <c r="A181" s="24">
         <v>18</v>
       </c>
-      <c r="B181" s="61">
+      <c r="B181" s="59">
         <v>12</v>
       </c>
       <c r="C181" s="24"/>
@@ -5455,7 +5449,7 @@
       <c r="A182" s="24">
         <v>19</v>
       </c>
-      <c r="B182" s="61">
+      <c r="B182" s="59">
         <v>13</v>
       </c>
       <c r="C182" s="24"/>
@@ -5465,7 +5459,7 @@
       <c r="A183" s="24">
         <v>20</v>
       </c>
-      <c r="B183" s="61">
+      <c r="B183" s="59">
         <v>14</v>
       </c>
       <c r="C183" s="24"/>
@@ -5475,7 +5469,7 @@
       <c r="A184" s="24">
         <v>21</v>
       </c>
-      <c r="B184" s="61">
+      <c r="B184" s="59">
         <v>14</v>
       </c>
       <c r="C184" s="24"/>
@@ -5485,7 +5479,7 @@
       <c r="A185" s="24">
         <v>22</v>
       </c>
-      <c r="B185" s="61">
+      <c r="B185" s="59">
         <v>14</v>
       </c>
       <c r="C185" s="24"/>
@@ -5495,7 +5489,7 @@
       <c r="A186" s="24">
         <v>23</v>
       </c>
-      <c r="B186" s="61">
+      <c r="B186" s="59">
         <v>15</v>
       </c>
       <c r="C186" s="24"/>
@@ -5503,7 +5497,7 @@
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A187" s="24"/>
-      <c r="B187" s="56"/>
+      <c r="B187" s="54"/>
       <c r="C187" s="24"/>
       <c r="G187" s="24"/>
     </row>
@@ -5513,189 +5507,189 @@
       <c r="C188" s="24"/>
       <c r="G188" s="24"/>
     </row>
-    <row r="189" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B189" s="65"/>
-      <c r="C189" s="54"/>
-      <c r="G189" s="54"/>
-    </row>
-    <row r="190" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="57" t="s">
+    <row r="189" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B189" s="63"/>
+      <c r="C189" s="52"/>
+      <c r="G189" s="52"/>
+    </row>
+    <row r="190" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="55" t="s">
         <v>107</v>
       </c>
-      <c r="B190" s="65"/>
-      <c r="C190" s="54"/>
-      <c r="G190" s="54"/>
-    </row>
-    <row r="191" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A191" s="57" t="s">
+      <c r="B190" s="63"/>
+      <c r="C190" s="52"/>
+      <c r="G190" s="52"/>
+    </row>
+    <row r="191" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A191" s="55" t="s">
         <v>93</v>
       </c>
-      <c r="B191" s="65" t="s">
+      <c r="B191" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="C191" s="54"/>
-      <c r="G191" s="54"/>
-    </row>
-    <row r="192" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="65">
-        <v>0</v>
-      </c>
-      <c r="B192" s="65">
-        <v>1</v>
-      </c>
-      <c r="C192" s="65">
+      <c r="C191" s="52"/>
+      <c r="G191" s="52"/>
+    </row>
+    <row r="192" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A192" s="63">
+        <v>0</v>
+      </c>
+      <c r="B192" s="63">
+        <v>1</v>
+      </c>
+      <c r="C192" s="63">
         <v>2</v>
       </c>
-      <c r="D192" s="65">
+      <c r="D192" s="63">
         <v>3</v>
       </c>
-      <c r="E192" s="65">
+      <c r="E192" s="63">
         <v>4</v>
       </c>
-      <c r="G192" s="54"/>
-    </row>
-    <row r="193" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A193" s="65">
-        <v>1</v>
-      </c>
-      <c r="B193" s="56">
+      <c r="G192" s="52"/>
+    </row>
+    <row r="193" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A193" s="63">
+        <v>1</v>
+      </c>
+      <c r="B193" s="54">
         <v>4</v>
       </c>
-      <c r="C193" s="65">
+      <c r="C193" s="63">
         <v>5</v>
       </c>
-      <c r="D193" s="65">
+      <c r="D193" s="63">
         <v>6</v>
       </c>
-      <c r="G193" s="54"/>
-    </row>
-    <row r="194" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A194" s="65">
+      <c r="G193" s="52"/>
+    </row>
+    <row r="194" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A194" s="63">
         <v>2</v>
       </c>
-      <c r="B194" s="56">
-        <v>0</v>
-      </c>
-      <c r="C194" s="65"/>
-      <c r="D194" s="65"/>
-      <c r="G194" s="54"/>
-    </row>
-    <row r="195" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A195" s="65">
+      <c r="B194" s="54">
+        <v>0</v>
+      </c>
+      <c r="C194" s="63"/>
+      <c r="D194" s="63"/>
+      <c r="G194" s="52"/>
+    </row>
+    <row r="195" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A195" s="63">
         <v>3</v>
       </c>
-      <c r="B195" s="56">
-        <v>0</v>
-      </c>
-      <c r="C195" s="65"/>
-      <c r="D195" s="65"/>
-      <c r="G195" s="54"/>
-    </row>
-    <row r="196" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A196" s="65">
+      <c r="B195" s="54">
+        <v>0</v>
+      </c>
+      <c r="C195" s="63"/>
+      <c r="D195" s="63"/>
+      <c r="G195" s="52"/>
+    </row>
+    <row r="196" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="63">
         <v>4</v>
       </c>
-      <c r="B196" s="56">
+      <c r="B196" s="54">
         <v>7</v>
       </c>
-      <c r="C196" s="65"/>
-      <c r="D196" s="65"/>
-      <c r="G196" s="54"/>
-    </row>
-    <row r="197" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="65">
+      <c r="C196" s="63"/>
+      <c r="D196" s="63"/>
+      <c r="G196" s="52"/>
+    </row>
+    <row r="197" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A197" s="63">
         <v>5</v>
       </c>
-      <c r="B197" s="56">
+      <c r="B197" s="54">
         <v>11</v>
       </c>
-      <c r="C197" s="65"/>
-      <c r="D197" s="65"/>
-      <c r="G197" s="54"/>
-    </row>
-    <row r="198" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="65">
+      <c r="C197" s="63"/>
+      <c r="D197" s="63"/>
+      <c r="G197" s="52"/>
+    </row>
+    <row r="198" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="63">
         <v>6</v>
       </c>
-      <c r="B198" s="56">
-        <v>0</v>
-      </c>
-      <c r="C198" s="65"/>
-      <c r="D198" s="65"/>
-      <c r="G198" s="54"/>
-    </row>
-    <row r="199" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="65">
+      <c r="B198" s="54">
+        <v>0</v>
+      </c>
+      <c r="C198" s="63"/>
+      <c r="D198" s="63"/>
+      <c r="G198" s="52"/>
+    </row>
+    <row r="199" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A199" s="63">
         <v>7</v>
       </c>
-      <c r="B199" s="56">
+      <c r="B199" s="54">
         <v>8</v>
       </c>
-      <c r="C199" s="65"/>
-      <c r="D199" s="65"/>
-      <c r="G199" s="54"/>
-    </row>
-    <row r="200" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="65">
+      <c r="C199" s="63"/>
+      <c r="D199" s="63"/>
+      <c r="G199" s="52"/>
+    </row>
+    <row r="200" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A200" s="63">
         <v>8</v>
       </c>
-      <c r="B200" s="56">
+      <c r="B200" s="54">
         <v>9</v>
       </c>
-      <c r="C200" s="65"/>
-      <c r="D200" s="65"/>
-      <c r="G200" s="54"/>
-    </row>
-    <row r="201" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="65">
+      <c r="C200" s="63"/>
+      <c r="D200" s="63"/>
+      <c r="G200" s="52"/>
+    </row>
+    <row r="201" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="63">
         <v>9</v>
       </c>
-      <c r="B201" s="56">
+      <c r="B201" s="54">
         <v>10</v>
       </c>
-      <c r="C201" s="65"/>
-      <c r="D201" s="65"/>
-      <c r="G201" s="54"/>
-    </row>
-    <row r="202" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="65">
+      <c r="C201" s="63"/>
+      <c r="D201" s="63"/>
+      <c r="G201" s="52"/>
+    </row>
+    <row r="202" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A202" s="63">
         <v>10</v>
       </c>
-      <c r="B202" s="56">
-        <v>0</v>
-      </c>
-      <c r="C202" s="65"/>
-      <c r="D202" s="65"/>
-      <c r="G202" s="54"/>
-    </row>
-    <row r="203" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A203" s="65">
+      <c r="B202" s="54">
+        <v>0</v>
+      </c>
+      <c r="C202" s="63"/>
+      <c r="D202" s="63"/>
+      <c r="G202" s="52"/>
+    </row>
+    <row r="203" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A203" s="63">
         <v>11</v>
       </c>
-      <c r="B203" s="56">
+      <c r="B203" s="54">
         <v>12</v>
       </c>
-      <c r="C203" s="65"/>
-      <c r="D203" s="65"/>
-      <c r="G203" s="54"/>
-    </row>
-    <row r="204" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A204" s="65">
+      <c r="C203" s="63"/>
+      <c r="D203" s="63"/>
+      <c r="G203" s="52"/>
+    </row>
+    <row r="204" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A204" s="63">
         <v>12</v>
       </c>
-      <c r="B204" s="56">
-        <v>0</v>
-      </c>
-      <c r="C204" s="65"/>
-      <c r="D204" s="65"/>
-      <c r="G204" s="54"/>
-    </row>
-    <row r="205" spans="1:7" s="57" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="65"/>
-      <c r="B205" s="56"/>
-      <c r="C205" s="65"/>
-      <c r="D205" s="65"/>
-      <c r="G205" s="54"/>
+      <c r="B204" s="54">
+        <v>0</v>
+      </c>
+      <c r="C204" s="63"/>
+      <c r="D204" s="63"/>
+      <c r="G204" s="52"/>
+    </row>
+    <row r="205" spans="1:7" s="55" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A205" s="63"/>
+      <c r="B205" s="54"/>
+      <c r="C205" s="63"/>
+      <c r="D205" s="63"/>
+      <c r="G205" s="52"/>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A206" s="18"/>
@@ -6255,7 +6249,7 @@
       <c r="A270">
         <v>13</v>
       </c>
-      <c r="B270" s="60">
+      <c r="B270" s="58">
         <v>1</v>
       </c>
       <c r="I270" s="18"/>
@@ -6264,7 +6258,7 @@
       <c r="A271">
         <v>14</v>
       </c>
-      <c r="B271" s="60">
+      <c r="B271" s="58">
         <v>1</v>
       </c>
       <c r="I271" s="18"/>
@@ -6273,7 +6267,7 @@
       <c r="A272">
         <v>15</v>
       </c>
-      <c r="B272" s="60">
+      <c r="B272" s="58">
         <v>1</v>
       </c>
       <c r="I272" s="18"/>
@@ -6282,7 +6276,7 @@
       <c r="A273">
         <v>16</v>
       </c>
-      <c r="B273" s="60">
+      <c r="B273" s="58">
         <v>1</v>
       </c>
       <c r="I273" s="18"/>
@@ -6291,7 +6285,7 @@
       <c r="A274">
         <v>17</v>
       </c>
-      <c r="B274" s="60">
+      <c r="B274" s="58">
         <v>1</v>
       </c>
       <c r="I274" s="18"/>
@@ -6300,7 +6294,7 @@
       <c r="A275">
         <v>18</v>
       </c>
-      <c r="B275" s="60">
+      <c r="B275" s="58">
         <v>1</v>
       </c>
       <c r="I275" s="18"/>
@@ -6309,7 +6303,7 @@
       <c r="A276">
         <v>19</v>
       </c>
-      <c r="B276" s="60">
+      <c r="B276" s="58">
         <v>1</v>
       </c>
       <c r="I276" s="18"/>
@@ -6318,7 +6312,7 @@
       <c r="A277">
         <v>20</v>
       </c>
-      <c r="B277" s="60">
+      <c r="B277" s="58">
         <v>2</v>
       </c>
       <c r="I277" s="18"/>
@@ -6327,7 +6321,7 @@
       <c r="A278">
         <v>21</v>
       </c>
-      <c r="B278" s="60">
+      <c r="B278" s="58">
         <v>2</v>
       </c>
       <c r="I278" s="18"/>
@@ -6336,7 +6330,7 @@
       <c r="A279">
         <v>22</v>
       </c>
-      <c r="B279" s="60">
+      <c r="B279" s="58">
         <v>1</v>
       </c>
       <c r="I279" s="18"/>
@@ -6466,7 +6460,7 @@
       <c r="A297">
         <v>13</v>
       </c>
-      <c r="B297" s="60">
+      <c r="B297" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6474,7 +6468,7 @@
       <c r="A298">
         <v>14</v>
       </c>
-      <c r="B298" s="60">
+      <c r="B298" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6482,7 +6476,7 @@
       <c r="A299">
         <v>15</v>
       </c>
-      <c r="B299" s="60">
+      <c r="B299" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6490,7 +6484,7 @@
       <c r="A300">
         <v>16</v>
       </c>
-      <c r="B300" s="60">
+      <c r="B300" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6498,7 +6492,7 @@
       <c r="A301">
         <v>17</v>
       </c>
-      <c r="B301" s="60">
+      <c r="B301" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6506,7 +6500,7 @@
       <c r="A302">
         <v>18</v>
       </c>
-      <c r="B302" s="60">
+      <c r="B302" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6514,7 +6508,7 @@
       <c r="A303">
         <v>19</v>
       </c>
-      <c r="B303" s="60">
+      <c r="B303" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6522,7 +6516,7 @@
       <c r="A304">
         <v>20</v>
       </c>
-      <c r="B304" s="60">
+      <c r="B304" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6530,7 +6524,7 @@
       <c r="A305">
         <v>21</v>
       </c>
-      <c r="B305" s="60">
+      <c r="B305" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6538,7 +6532,7 @@
       <c r="A306">
         <v>22</v>
       </c>
-      <c r="B306" s="60">
+      <c r="B306" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6546,7 +6540,7 @@
       <c r="A307">
         <v>23</v>
       </c>
-      <c r="B307" s="60">
+      <c r="B307" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6663,7 +6657,7 @@
       <c r="A324">
         <v>13</v>
       </c>
-      <c r="B324" s="60">
+      <c r="B324" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6671,7 +6665,7 @@
       <c r="A325">
         <v>14</v>
       </c>
-      <c r="B325" s="60">
+      <c r="B325" s="58">
         <v>0</v>
       </c>
     </row>
@@ -6679,7 +6673,7 @@
       <c r="A326">
         <v>15</v>
       </c>
-      <c r="B326" s="60">
+      <c r="B326" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6687,7 +6681,7 @@
       <c r="A327">
         <v>16</v>
       </c>
-      <c r="B327" s="60">
+      <c r="B327" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6695,7 +6689,7 @@
       <c r="A328">
         <v>17</v>
       </c>
-      <c r="B328" s="60">
+      <c r="B328" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6703,7 +6697,7 @@
       <c r="A329">
         <v>18</v>
       </c>
-      <c r="B329" s="60">
+      <c r="B329" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6711,7 +6705,7 @@
       <c r="A330">
         <v>19</v>
       </c>
-      <c r="B330" s="60">
+      <c r="B330" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6719,7 +6713,7 @@
       <c r="A331">
         <v>20</v>
       </c>
-      <c r="B331" s="60">
+      <c r="B331" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6727,7 +6721,7 @@
       <c r="A332">
         <v>21</v>
       </c>
-      <c r="B332" s="60">
+      <c r="B332" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6735,7 +6729,7 @@
       <c r="A333">
         <v>22</v>
       </c>
-      <c r="B333" s="60">
+      <c r="B333" s="58">
         <v>1</v>
       </c>
     </row>
@@ -6743,7 +6737,7 @@
       <c r="A334">
         <v>23</v>
       </c>
-      <c r="B334" s="60">
+      <c r="B334" s="58">
         <v>2</v>
       </c>
     </row>
@@ -6991,189 +6985,189 @@
       </c>
     </row>
     <row r="352" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A352" s="60">
+      <c r="A352" s="58">
         <v>13</v>
       </c>
-      <c r="B352" s="60">
+      <c r="B352" s="58">
         <v>-1</v>
       </c>
-      <c r="C352" s="60">
+      <c r="C352" s="58">
         <v>19</v>
       </c>
-      <c r="D352" s="60">
+      <c r="D352" s="58">
         <v>-1</v>
       </c>
-      <c r="E352" s="60">
+      <c r="E352" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="353" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A353" s="60">
+      <c r="A353" s="58">
         <v>14</v>
       </c>
-      <c r="B353" s="60">
+      <c r="B353" s="58">
         <v>20</v>
       </c>
-      <c r="C353" s="60">
+      <c r="C353" s="58">
         <v>21</v>
       </c>
-      <c r="D353" s="60">
+      <c r="D353" s="58">
         <v>22</v>
       </c>
-      <c r="E353" s="60">
+      <c r="E353" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="354" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A354" s="60">
+      <c r="A354" s="58">
         <v>15</v>
       </c>
-      <c r="B354" s="60">
+      <c r="B354" s="58">
         <v>-1</v>
       </c>
-      <c r="C354" s="60">
+      <c r="C354" s="58">
         <v>23</v>
       </c>
-      <c r="D354" s="60">
+      <c r="D354" s="58">
         <v>-1</v>
       </c>
-      <c r="E354" s="60">
+      <c r="E354" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="355" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A355" s="60">
+      <c r="A355" s="58">
         <v>16</v>
       </c>
-      <c r="B355" s="60">
+      <c r="B355" s="58">
         <v>-1</v>
       </c>
-      <c r="C355" s="60">
-        <v>0</v>
-      </c>
-      <c r="D355" s="60">
+      <c r="C355" s="58">
+        <v>0</v>
+      </c>
+      <c r="D355" s="58">
         <v>-1</v>
       </c>
-      <c r="E355" s="60">
+      <c r="E355" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="356" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A356" s="60">
+      <c r="A356" s="58">
         <v>17</v>
       </c>
-      <c r="B356" s="60">
+      <c r="B356" s="58">
         <v>-1</v>
       </c>
-      <c r="C356" s="60">
-        <v>0</v>
-      </c>
-      <c r="D356" s="60">
+      <c r="C356" s="58">
+        <v>0</v>
+      </c>
+      <c r="D356" s="58">
         <v>-1</v>
       </c>
-      <c r="E356" s="60">
+      <c r="E356" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="357" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A357" s="60">
+      <c r="A357" s="58">
         <v>18</v>
       </c>
-      <c r="B357" s="60">
+      <c r="B357" s="58">
         <v>-1</v>
       </c>
-      <c r="C357" s="60">
-        <v>0</v>
-      </c>
-      <c r="D357" s="60">
+      <c r="C357" s="58">
+        <v>0</v>
+      </c>
+      <c r="D357" s="58">
         <v>-1</v>
       </c>
-      <c r="E357" s="60">
+      <c r="E357" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="358" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A358" s="60">
+      <c r="A358" s="58">
         <v>19</v>
       </c>
-      <c r="B358" s="60">
+      <c r="B358" s="58">
         <v>-1</v>
       </c>
-      <c r="C358" s="60">
-        <v>0</v>
-      </c>
-      <c r="D358" s="60">
+      <c r="C358" s="58">
+        <v>0</v>
+      </c>
+      <c r="D358" s="58">
         <v>-1</v>
       </c>
-      <c r="E358" s="60">
+      <c r="E358" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="359" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A359" s="60">
+      <c r="A359" s="58">
         <v>20</v>
       </c>
-      <c r="B359" s="60">
+      <c r="B359" s="58">
         <v>-1</v>
       </c>
-      <c r="C359" s="60">
+      <c r="C359" s="58">
         <v>-1</v>
       </c>
-      <c r="D359" s="60">
-        <v>0</v>
-      </c>
-      <c r="E359" s="60">
+      <c r="D359" s="58">
+        <v>0</v>
+      </c>
+      <c r="E359" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="360" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A360" s="60">
+      <c r="A360" s="58">
         <v>21</v>
       </c>
-      <c r="B360" s="60">
+      <c r="B360" s="58">
         <v>-1</v>
       </c>
-      <c r="C360" s="60">
+      <c r="C360" s="58">
         <v>-1</v>
       </c>
-      <c r="D360" s="60">
-        <v>0</v>
-      </c>
-      <c r="E360" s="60">
+      <c r="D360" s="58">
+        <v>0</v>
+      </c>
+      <c r="E360" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="361" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A361" s="60">
+      <c r="A361" s="58">
         <v>22</v>
       </c>
-      <c r="B361" s="60">
+      <c r="B361" s="58">
         <v>-1</v>
       </c>
-      <c r="C361" s="60">
-        <v>0</v>
-      </c>
-      <c r="D361" s="60">
+      <c r="C361" s="58">
+        <v>0</v>
+      </c>
+      <c r="D361" s="58">
         <v>-1</v>
       </c>
-      <c r="E361" s="60">
+      <c r="E361" s="58">
         <v>-1</v>
       </c>
     </row>
     <row r="362" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A362" s="60">
+      <c r="A362" s="58">
         <v>23</v>
       </c>
-      <c r="B362" s="60">
+      <c r="B362" s="58">
         <v>-1</v>
       </c>
-      <c r="C362" s="60">
+      <c r="C362" s="58">
         <v>-1</v>
       </c>
-      <c r="D362" s="60">
-        <v>0</v>
-      </c>
-      <c r="E362" s="60">
+      <c r="D362" s="58">
+        <v>0</v>
+      </c>
+      <c r="E362" s="58">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add HMI WiFi setup flow and WiFi settings tab
</commit_message>
<xml_diff>
--- a/Kaffeewaage.Logik.20250103.xlsx
+++ b/Kaffeewaage.Logik.20250103.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bernh\Documents\PlatformIO\Projects\KaffeewaageESP_SingleDose\KaffeewaageLilygoT-DisplayS3_20240212\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F11B8A-4F31-4EA4-A33E-9741DCDB480A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F869C583-3C7E-436F-BAA2-BF645713E811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{6093FCE1-E198-4E7B-9A9F-5F65F14DDFBD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="315">
   <si>
     <t>Input</t>
   </si>
@@ -665,34 +665,13 @@
 pageID=19</t>
   </si>
   <si>
-    <t>Muehle Reset?
-OK</t>
-  </si>
-  <si>
-    <t>Kaffeem. Reset?
-OK</t>
-  </si>
-  <si>
-    <t>Filterwechsel Reset?
-OK</t>
-  </si>
-  <si>
     <t>Mahlgewichte</t>
   </si>
   <si>
     <t>Shots</t>
   </si>
   <si>
-    <t>Gesamt
-Seit Reinigung
-OK</t>
-  </si>
-  <si>
     <t>IP-Adresse</t>
-  </si>
-  <si>
-    <t>IP-Adresse
-OK</t>
   </si>
   <si>
     <t>leer tara --&gt; set, Variable: Gefaess 2</t>
@@ -771,10 +750,6 @@
 pageID=21</t>
   </si>
   <si>
-    <t>IP-Adresse
-pageID=22</t>
-  </si>
-  <si>
     <t>Stoppuhr
 Nur Funktionsaufruf Tara
 menuItemID=2</t>
@@ -1163,6 +1138,59 @@
   <si>
     <t>Gefaess messen, Gefaess gemessen
 pageID=23</t>
+  </si>
+  <si>
+    <t>WLAN/Netzwerk</t>
+  </si>
+  <si>
+    <t>WLAN/Netzwerk
+pageID=22</t>
+  </si>
+  <si>
+    <t>WLAN neu verbinden
+pageID=24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit WLAN Waagen-
+Setup verbinden
+IP: 192.168.4.1 
+aufrufen
+Warten…
+Set Button ist hier ausgeblendet. Es wird automatisch bei Speichern über die WebUI auf die nächste Seite pageID26 gewechselt. pageID25 wird übersprungen. </t>
+  </si>
+  <si>
+    <t>WLAN gespeichert
+pageID=26</t>
+  </si>
+  <si>
+    <t>Daten gespeichert
+Neustart noetig
+WebUI oder HMI
+&gt; Neustart
+Set ist wieder eingeblendet</t>
+  </si>
+  <si>
+    <t>SSID:
+FRITZ!Box ….
+IP: ….
+&gt;Setup starten</t>
+  </si>
+  <si>
+    <t>Gesamt
+Seit Reinigung
+&gt;OK</t>
+  </si>
+  <si>
+    <t>Filterwechsel Reset?
+&gt;OK</t>
+  </si>
+  <si>
+    <t>Kaffeem. Reset?
+&gt;OK</t>
+  </si>
+  <si>
+    <t>Muehle Reset?
+&gt;OK</t>
   </si>
 </sst>
 </file>
@@ -2723,7 +2751,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA8C470F-6C58-48CC-9954-EE9382CE54CA}">
-  <dimension ref="A3:G36"/>
+  <dimension ref="A3:H36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
@@ -2757,95 +2785,95 @@
         <v>112</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="E5" s="48" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="F5" s="48" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="G5" s="48" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5"/>
       <c r="C6" s="28" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D6" s="35" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E6" s="45" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="5"/>
       <c r="C7" s="10"/>
       <c r="D7" s="35" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="5"/>
       <c r="C8" s="10"/>
       <c r="D8" s="35" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="5"/>
       <c r="C9" s="10"/>
       <c r="D9" s="35" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="5"/>
       <c r="C10" s="10"/>
       <c r="D10" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>216</v>
+      </c>
+      <c r="F10" s="50" t="s">
         <v>229</v>
-      </c>
-      <c r="E10" s="50" t="s">
-        <v>221</v>
-      </c>
-      <c r="F10" s="50" t="s">
-        <v>235</v>
       </c>
       <c r="G10" s="25"/>
     </row>
@@ -2855,10 +2883,10 @@
         <v>135</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F11" s="30" t="s">
         <v>188</v>
@@ -2869,7 +2897,7 @@
       <c r="B12" s="36"/>
       <c r="C12" s="39"/>
       <c r="D12" s="51" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="E12" s="40"/>
       <c r="F12" s="37"/>
@@ -2878,10 +2906,10 @@
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B13" s="36"/>
       <c r="C13" s="35" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E13" s="39"/>
       <c r="G13" s="34"/>
@@ -2890,7 +2918,7 @@
       <c r="B14" s="36"/>
       <c r="C14" s="41"/>
       <c r="D14" s="35" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="E14" s="39"/>
       <c r="G14" s="34"/>
@@ -2898,16 +2926,16 @@
     <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B15" s="36"/>
       <c r="C15" s="35" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="D15" s="51" t="s">
+        <v>224</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>225</v>
+      </c>
+      <c r="F15" s="51" t="s">
         <v>230</v>
-      </c>
-      <c r="E15" s="51" t="s">
-        <v>231</v>
-      </c>
-      <c r="F15" s="51" t="s">
-        <v>236</v>
       </c>
       <c r="G15" s="34"/>
     </row>
@@ -2915,139 +2943,149 @@
       <c r="B16" s="36"/>
       <c r="C16" s="39"/>
       <c r="D16" s="35" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E16" s="35" t="s">
         <v>194</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>201</v>
+        <v>314</v>
       </c>
       <c r="G16" s="34"/>
     </row>
-    <row r="17" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B17" s="36"/>
       <c r="C17" s="41"/>
       <c r="D17" s="39"/>
       <c r="E17" s="51" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="G17" s="34"/>
     </row>
-    <row r="18" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B18" s="36"/>
       <c r="C18" s="41"/>
       <c r="D18" s="35" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E18" s="35" t="s">
         <v>194</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>202</v>
+        <v>313</v>
       </c>
       <c r="G18" s="34"/>
     </row>
-    <row r="19" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B19" s="36"/>
       <c r="C19" s="41"/>
       <c r="D19" s="39"/>
       <c r="E19" s="51" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>200</v>
       </c>
       <c r="G19" s="34"/>
     </row>
-    <row r="20" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B20" s="36"/>
       <c r="C20" s="41"/>
       <c r="D20" s="35" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E20" s="35" t="s">
         <v>194</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>203</v>
+        <v>312</v>
       </c>
       <c r="G20" s="34"/>
     </row>
-    <row r="21" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B21" s="36"/>
       <c r="C21" s="41"/>
       <c r="D21" s="39"/>
       <c r="E21" s="51" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="F21" s="51" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="G21" s="34"/>
     </row>
-    <row r="22" spans="2:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="36"/>
       <c r="C22" s="42"/>
       <c r="D22" s="35" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F22" s="35" t="s">
-        <v>206</v>
+        <v>311</v>
       </c>
       <c r="G22" s="34"/>
     </row>
-    <row r="23" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B23" s="36"/>
       <c r="C23" s="56"/>
       <c r="D23" s="41"/>
       <c r="E23" s="41"/>
       <c r="F23" s="51" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="G23" s="34"/>
     </row>
-    <row r="24" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B24" s="36"/>
       <c r="C24" s="56"/>
       <c r="D24" s="41"/>
       <c r="E24" s="35" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F24" s="57" t="s">
-        <v>206</v>
+        <v>311</v>
       </c>
       <c r="G24" s="34"/>
     </row>
-    <row r="25" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
       <c r="C25" s="56"/>
       <c r="D25" s="56"/>
       <c r="E25" s="41"/>
       <c r="F25" s="51" t="s">
-        <v>224</v>
-      </c>
-      <c r="G25" s="34"/>
-    </row>
-    <row r="26" spans="2:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+        <v>305</v>
+      </c>
+      <c r="G25" s="51" t="s">
+        <v>306</v>
+      </c>
+      <c r="H25" s="51" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="36"/>
       <c r="C26" s="56"/>
       <c r="D26" s="56"/>
       <c r="E26" s="35" t="s">
-        <v>207</v>
+        <v>304</v>
       </c>
       <c r="F26" s="35" t="s">
-        <v>208</v>
-      </c>
-      <c r="G26" s="34"/>
-    </row>
-    <row r="27" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>310</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="H26" s="35" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B27" s="27" t="s">
         <v>136</v>
       </c>
@@ -3059,52 +3097,52 @@
       <c r="F27" s="9"/>
       <c r="G27" s="16"/>
     </row>
-    <row r="28" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B28" s="6"/>
       <c r="C28" s="43" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="11"/>
       <c r="F28" s="11"/>
       <c r="G28" s="13"/>
     </row>
-    <row r="29" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B29" s="6"/>
       <c r="C29" s="43" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="11"/>
       <c r="F29" s="11"/>
       <c r="G29" s="13"/>
     </row>
-    <row r="30" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B30" s="6"/>
       <c r="C30" s="43" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="11"/>
       <c r="F30" s="11"/>
       <c r="G30" s="13"/>
     </row>
-    <row r="31" spans="2:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:8" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6"/>
       <c r="C31" s="29" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="14"/>
       <c r="F31" s="14"/>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="2:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:8" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="27" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C32" s="51" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
@@ -3116,7 +3154,7 @@
         <v>137</v>
       </c>
       <c r="C33" s="51" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
@@ -3126,7 +3164,7 @@
     <row r="34" spans="2:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="7"/>
       <c r="C34" s="29" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
@@ -3230,13 +3268,13 @@
         <v>80</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>81</v>
@@ -3268,7 +3306,7 @@
         <v>83</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="H7" s="18"/>
     </row>
@@ -3298,13 +3336,13 @@
         <v>80</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>85</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="H9" s="18"/>
     </row>
@@ -3330,7 +3368,7 @@
         <v>87</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="H11" s="18"/>
     </row>
@@ -3343,7 +3381,7 @@
         <v>88</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="H12" s="18"/>
     </row>
@@ -3358,13 +3396,13 @@
         <v>80</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H13" s="18"/>
     </row>
@@ -3373,19 +3411,19 @@
         <v>83</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H14" s="18"/>
     </row>
@@ -3394,19 +3432,19 @@
         <v>84</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="D15" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H15" s="18"/>
     </row>
@@ -3415,7 +3453,7 @@
         <v>85</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>81</v>
@@ -3427,7 +3465,7 @@
         <v>89</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="H16" s="18"/>
     </row>
@@ -3448,7 +3486,7 @@
         <v>90</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="H17" s="18"/>
     </row>
@@ -3457,7 +3495,7 @@
         <v>87</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="D18" s="19" t="s">
         <v>81</v>
@@ -3469,7 +3507,7 @@
         <v>80</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H18" s="18"/>
     </row>
@@ -3478,7 +3516,7 @@
         <v>88</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>81</v>
@@ -3490,7 +3528,7 @@
         <v>91</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="H19" s="18"/>
     </row>
@@ -3538,19 +3576,19 @@
         <v>89</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="D23" s="19" t="s">
         <v>85</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>191</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="H23" s="18"/>
     </row>
@@ -3559,7 +3597,7 @@
         <v>90</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>86</v>
@@ -3580,19 +3618,19 @@
         <v>91</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>88</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>193</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="H25" s="18"/>
     </row>
@@ -3607,10 +3645,10 @@
         <v>88</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>187</v>
@@ -3628,10 +3666,10 @@
         <v>88</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>186</v>
@@ -3649,13 +3687,13 @@
         <v>88</v>
       </c>
       <c r="E28" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>270</v>
-      </c>
       <c r="G28" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H28" s="18"/>
     </row>
@@ -3665,10 +3703,10 @@
       <c r="D29" s="19"/>
       <c r="E29" s="20"/>
       <c r="F29" s="4" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H29" s="18"/>
     </row>
@@ -3678,10 +3716,10 @@
       <c r="D30" s="19"/>
       <c r="E30" s="20"/>
       <c r="F30" s="19" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H30" s="18"/>
     </row>
@@ -3690,19 +3728,19 @@
         <v>191</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="D31" s="19" t="s">
         <v>89</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="H31" s="18"/>
     </row>
@@ -3717,13 +3755,13 @@
         <v>90</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="F32" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H32" s="4"/>
     </row>
@@ -3732,25 +3770,25 @@
         <v>193</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>91</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="F33" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B34" s="19" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>187</v>
@@ -3765,13 +3803,13 @@
         <v>80</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H34" s="4"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B35" s="19" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>186</v>
@@ -3786,16 +3824,16 @@
         <v>80</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B36" s="4" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D36" s="19" t="s">
         <v>190</v>
@@ -3807,16 +3845,16 @@
         <v>80</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H36" s="4"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B37" s="4" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D37" s="19" t="s">
         <v>190</v>
@@ -3828,16 +3866,16 @@
         <v>80</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B38" s="19" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D38" s="19" t="s">
         <v>190</v>
@@ -3849,28 +3887,28 @@
         <v>80</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H38" s="4"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B39" s="4" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="D39" s="19" t="s">
         <v>191</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="F39" s="19" t="s">
         <v>80</v>
       </c>
       <c r="G39" s="20" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H39" s="4"/>
     </row>
@@ -4005,7 +4043,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="24" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C51" s="24"/>
       <c r="G51" s="24"/>
@@ -4038,7 +4076,7 @@
         <v>3</v>
       </c>
       <c r="B54" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C54" s="24"/>
       <c r="G54" s="24"/>
@@ -4048,7 +4086,7 @@
         <v>4</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C55" s="24"/>
       <c r="G55" s="24"/>
@@ -4058,7 +4096,7 @@
         <v>5</v>
       </c>
       <c r="B56" s="24" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C56" s="24"/>
       <c r="G56" s="24"/>
@@ -4078,7 +4116,7 @@
         <v>7</v>
       </c>
       <c r="B58" s="24" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C58" s="24"/>
       <c r="G58" s="24"/>
@@ -4088,7 +4126,7 @@
         <v>8</v>
       </c>
       <c r="B59" s="24" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C59" s="24"/>
       <c r="G59" s="24"/>
@@ -4098,7 +4136,7 @@
         <v>9</v>
       </c>
       <c r="B60" s="24" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="C60" s="24"/>
       <c r="G60" s="24"/>
@@ -4157,7 +4195,7 @@
         <v>15</v>
       </c>
       <c r="B66" s="24" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C66" s="24"/>
       <c r="G66" s="24"/>
@@ -4207,7 +4245,7 @@
         <v>20</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C71" s="24"/>
       <c r="G71" s="24"/>
@@ -4217,7 +4255,7 @@
         <v>21</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C72" s="24"/>
       <c r="G72" s="24"/>
@@ -4227,7 +4265,7 @@
         <v>22</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C73" s="24"/>
       <c r="G73" s="24"/>
@@ -4237,7 +4275,7 @@
         <v>23</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C74" s="24"/>
       <c r="G74" s="24"/>
@@ -4288,7 +4326,7 @@
         <v>72</v>
       </c>
       <c r="D81" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="E81" s="24" t="s">
         <v>126</v>
@@ -4300,16 +4338,16 @@
         <v>1</v>
       </c>
       <c r="B82" s="60" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C82" s="60" t="s">
         <v>127</v>
       </c>
       <c r="D82" s="58" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="E82" s="60" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="G82" s="24"/>
     </row>
@@ -4321,13 +4359,13 @@
         <v>129</v>
       </c>
       <c r="C83" s="58" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="D83" s="58" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E83" s="58" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="G83" s="24"/>
     </row>
@@ -4360,7 +4398,7 @@
         <v>72</v>
       </c>
       <c r="D85" s="58" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="E85" s="60" t="s">
         <v>126</v>
@@ -4372,16 +4410,16 @@
         <v>5</v>
       </c>
       <c r="B86" s="60" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C86" s="60" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="D86" s="58" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="E86" s="60" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G86" s="24"/>
     </row>
@@ -4408,10 +4446,10 @@
         <v>7</v>
       </c>
       <c r="B88" s="60" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="C88" s="60" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D88" s="60" t="s">
         <v>128</v>
@@ -4444,7 +4482,7 @@
         <v>9</v>
       </c>
       <c r="B90" s="60" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C90" s="60" t="s">
         <v>130</v>
@@ -4462,10 +4500,10 @@
         <v>10</v>
       </c>
       <c r="B91" s="60" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C91" s="60" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="D91" s="60" t="s">
         <v>128</v>
@@ -4480,7 +4518,7 @@
         <v>11</v>
       </c>
       <c r="B92" s="60" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C92" s="60" t="s">
         <v>196</v>
@@ -4498,7 +4536,7 @@
         <v>12</v>
       </c>
       <c r="B93" s="60" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C93" s="60" t="s">
         <v>196</v>
@@ -4516,7 +4554,7 @@
         <v>13</v>
       </c>
       <c r="B94" s="60" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C94" s="60" t="s">
         <v>196</v>
@@ -4530,13 +4568,13 @@
         <v>14</v>
       </c>
       <c r="B95" s="60" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C95" s="60" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D95" s="60" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="E95" s="60" t="s">
         <v>128</v>
@@ -4548,10 +4586,10 @@
         <v>15</v>
       </c>
       <c r="B96" s="60" t="s">
+        <v>285</v>
+      </c>
+      <c r="C96" s="60" t="s">
         <v>291</v>
-      </c>
-      <c r="C96" s="60" t="s">
-        <v>297</v>
       </c>
       <c r="D96" s="60" t="s">
         <v>128</v>
@@ -4566,7 +4604,7 @@
         <v>16</v>
       </c>
       <c r="B97" s="60" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C97" s="60" t="s">
         <v>146</v>
@@ -4584,7 +4622,7 @@
         <v>17</v>
       </c>
       <c r="B98" s="62" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="C98" s="60" t="s">
         <v>146</v>
@@ -4602,7 +4640,7 @@
         <v>18</v>
       </c>
       <c r="B99" s="62" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C99" s="60" t="s">
         <v>146</v>
@@ -4620,7 +4658,7 @@
         <v>19</v>
       </c>
       <c r="B100" s="62" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C100" s="60" t="s">
         <v>146</v>
@@ -4638,10 +4676,10 @@
         <v>20</v>
       </c>
       <c r="B101" s="62" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="C101" s="60" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D101" s="60" t="s">
         <v>146</v>
@@ -4656,10 +4694,10 @@
         <v>21</v>
       </c>
       <c r="B102" s="62" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="C102" s="60" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="D102" s="60" t="s">
         <v>146</v>
@@ -4674,7 +4712,7 @@
         <v>22</v>
       </c>
       <c r="B103" s="62" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C103" s="60" t="s">
         <v>146</v>
@@ -4692,10 +4730,10 @@
         <v>23</v>
       </c>
       <c r="B104" s="60" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="C104" s="60" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="D104" s="60" t="s">
         <v>146</v>
@@ -4735,7 +4773,7 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="G108" s="24"/>
     </row>
@@ -4759,7 +4797,7 @@
         <v>1</v>
       </c>
       <c r="D110" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="G110" s="24"/>
     </row>

</xml_diff>